<commit_message>
chore: update daily job tracker
</commit_message>
<xml_diff>
--- a/data/archive/2026-09-24.xlsx
+++ b/data/archive/2026-09-24.xlsx
@@ -645,7 +645,7 @@
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 16:25 UTC</t>
+          <t>2026-09-24 17:06 UTC</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
@@ -732,7 +732,7 @@
       </c>
       <c r="N3" s="4" t="inlineStr">
         <is>
-          <t>2026-09-24 16:25 UTC</t>
+          <t>2026-09-24 17:07 UTC</t>
         </is>
       </c>
       <c r="O3" s="4" t="inlineStr">
@@ -815,7 +815,7 @@
       </c>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-24 16:26 UTC</t>
+          <t>2026-09-24 17:07 UTC</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">

</xml_diff>